<commit_message>
Update VDS factors for each sector.xlsx
</commit_message>
<xml_diff>
--- a/clustering/sepsectors/VDS factors for each sector.xlsx
+++ b/clustering/sepsectors/VDS factors for each sector.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="43">
   <si>
     <t>Сектор</t>
   </si>
@@ -121,6 +121,33 @@
   </si>
   <si>
     <t>ДОБЫЧА ПОЛЕЗНЫХ ИСКОПАЕМЫХ</t>
+  </si>
+  <si>
+    <t>Оптимизация извлечения полезных ископаемых</t>
+  </si>
+  <si>
+    <t>Геолого-геофизическое моделирование и прогнозирование</t>
+  </si>
+  <si>
+    <t>Оптимизация производственных процессов и режимов добычи</t>
+  </si>
+  <si>
+    <t>Повышение производительности и эффективности оборудования</t>
+  </si>
+  <si>
+    <t>Снижение ресурсоёмкости и себестоимости добычи</t>
+  </si>
+  <si>
+    <t>Управление рисками и обеспечение промышленной безопасности</t>
+  </si>
+  <si>
+    <t>Повышение качества и концентрации добываемого сырья</t>
+  </si>
+  <si>
+    <t>Оптимизация логистики и инфраструктуры добычи</t>
+  </si>
+  <si>
+    <t>Комплексное освоение месторождений и сокращение потерь</t>
   </si>
 </sst>
 </file>
@@ -145,18 +172,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -182,6 +203,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF33CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -195,15 +228,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -218,12 +251,20 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF33CC"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -503,7 +544,7 @@
   <cols>
     <col min="1" max="1" width="45.85546875" customWidth="1"/>
     <col min="2" max="2" width="73.42578125" customWidth="1"/>
-    <col min="3" max="3" width="58.5703125" customWidth="1"/>
+    <col min="3" max="3" width="65.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -529,51 +570,80 @@
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="6" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>4</v>
       </c>
+      <c r="C4" s="5" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>5</v>
       </c>
+      <c r="C5" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="6" t="s">
         <v>6</v>
       </c>
+      <c r="C6" s="5" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>7</v>
       </c>
+      <c r="C7" s="5" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>8</v>
       </c>
+      <c r="C8" s="5" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="5" t="s">
         <v>9</v>
       </c>
+      <c r="C9" s="8" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="5" t="s">
         <v>10</v>
       </c>
+      <c r="C10" s="5" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="6" t="s">
         <v>11</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C12" s="5" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -585,74 +655,74 @@
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B18" s="7" t="s">
+      <c r="B18" s="6" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="7" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="5" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="3" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
+      <c r="A22" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="B22" s="8" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="5" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="4" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="5" t="s">
+      <c r="A25" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="4" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="5" t="s">
+      <c r="A26" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="4" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>